<commit_message>
fix: Update GitHub Action workflows to output all 4 test category Excel reports in every run
</commit_message>
<xml_diff>
--- a/Excel_Reports/All_Test_Results_Master.xlsx
+++ b/Excel_Reports/All_Test_Results_Master.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14029" uniqueCount="3290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14029" uniqueCount="3291">
   <si>
     <t>#</t>
   </si>
@@ -7529,7 +7529,7 @@
     <t>[TC-SEC-001] Automated Assertion for SQL Injection Input Sanitization #1</t>
   </si>
   <si>
-    <t>2026-08-20T08:05:48.219Z</t>
+    <t>2026-08-20T08:19:48.920Z</t>
   </si>
   <si>
     <t>[TC-SEC-002] Automated Assertion for SQL Injection Input Sanitization #2</t>
@@ -7925,7 +7925,7 @@
     <t>100</t>
   </si>
   <si>
-    <t>20/8/2026, 1:35:48 pm</t>
+    <t>20/8/2026, 1:49:48 pm</t>
   </si>
   <si>
     <t>Total Vulnerability Tests</t>
@@ -9876,6 +9876,9 @@
   </si>
   <si>
     <t>Avg Response (ms)</t>
+  </si>
+  <si>
+    <t>20/8/2026, 1:49:49 pm</t>
   </si>
   <si>
     <t>Total Unique Load Scenarios</t>
@@ -35856,12 +35859,12 @@
         <v>1360</v>
       </c>
       <c r="B2" t="s">
-        <v>2634</v>
+        <v>3285</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3285</v>
+        <v>3286</v>
       </c>
       <c r="B3">
         <v>300</v>
@@ -35869,7 +35872,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3286</v>
+        <v>3287</v>
       </c>
       <c r="B4">
         <v>300</v>
@@ -35877,7 +35880,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3287</v>
+        <v>3288</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -35893,10 +35896,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>3288</v>
+        <v>3289</v>
       </c>
       <c r="B7" t="s">
-        <v>3289</v>
+        <v>3290</v>
       </c>
     </row>
   </sheetData>
@@ -64489,7 +64492,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F2" t="s">
         <v>2502</v>
@@ -64535,7 +64538,7 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F4" t="s">
         <v>2502</v>
@@ -64558,7 +64561,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F5" t="s">
         <v>2502</v>
@@ -64581,7 +64584,7 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F6" t="s">
         <v>2502</v>
@@ -64604,7 +64607,7 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
         <v>2502</v>
@@ -64627,7 +64630,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F8" t="s">
         <v>2502</v>
@@ -64650,7 +64653,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F9" t="s">
         <v>2502</v>
@@ -64673,7 +64676,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
         <v>2502</v>
@@ -64696,7 +64699,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
         <v>2502</v>
@@ -64719,7 +64722,7 @@
         <v>9</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F12" t="s">
         <v>2502</v>
@@ -64742,7 +64745,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F13" t="s">
         <v>2502</v>
@@ -64765,7 +64768,7 @@
         <v>9</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
         <v>2502</v>
@@ -64788,7 +64791,7 @@
         <v>9</v>
       </c>
       <c r="E15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F15" t="s">
         <v>2502</v>
@@ -64811,7 +64814,7 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F16" t="s">
         <v>2502</v>
@@ -64834,7 +64837,7 @@
         <v>9</v>
       </c>
       <c r="E17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="s">
         <v>2502</v>
@@ -64857,7 +64860,7 @@
         <v>9</v>
       </c>
       <c r="E18">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F18" t="s">
         <v>2502</v>
@@ -64880,7 +64883,7 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F19" t="s">
         <v>2502</v>
@@ -64903,7 +64906,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="s">
         <v>2502</v>
@@ -64926,7 +64929,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F21" t="s">
         <v>2502</v>
@@ -64949,7 +64952,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F22" t="s">
         <v>2502</v>
@@ -64972,7 +64975,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F23" t="s">
         <v>2502</v>
@@ -64995,7 +64998,7 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F24" t="s">
         <v>2502</v>
@@ -65018,7 +65021,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F25" t="s">
         <v>2502</v>
@@ -65041,7 +65044,7 @@
         <v>9</v>
       </c>
       <c r="E26">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F26" t="s">
         <v>2502</v>
@@ -65064,7 +65067,7 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F27" t="s">
         <v>2502</v>
@@ -65087,7 +65090,7 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="F28" t="s">
         <v>2502</v>
@@ -65110,7 +65113,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F29" t="s">
         <v>2502</v>
@@ -65133,7 +65136,7 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F30" t="s">
         <v>2502</v>
@@ -65156,7 +65159,7 @@
         <v>9</v>
       </c>
       <c r="E31">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F31" t="s">
         <v>2502</v>
@@ -65179,7 +65182,7 @@
         <v>9</v>
       </c>
       <c r="E32">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F32" t="s">
         <v>2502</v>
@@ -65202,7 +65205,7 @@
         <v>9</v>
       </c>
       <c r="E33">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F33" t="s">
         <v>2502</v>
@@ -65225,7 +65228,7 @@
         <v>9</v>
       </c>
       <c r="E34">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F34" t="s">
         <v>2502</v>
@@ -65248,7 +65251,7 @@
         <v>9</v>
       </c>
       <c r="E35">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F35" t="s">
         <v>2502</v>
@@ -65271,7 +65274,7 @@
         <v>9</v>
       </c>
       <c r="E36">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F36" t="s">
         <v>2502</v>
@@ -65294,7 +65297,7 @@
         <v>9</v>
       </c>
       <c r="E37">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F37" t="s">
         <v>2502</v>
@@ -65340,7 +65343,7 @@
         <v>9</v>
       </c>
       <c r="E39">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F39" t="s">
         <v>2502</v>
@@ -65363,7 +65366,7 @@
         <v>9</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="s">
         <v>2502</v>
@@ -65386,7 +65389,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
         <v>2502</v>
@@ -65409,7 +65412,7 @@
         <v>9</v>
       </c>
       <c r="E42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F42" t="s">
         <v>2502</v>
@@ -65455,7 +65458,7 @@
         <v>9</v>
       </c>
       <c r="E44">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F44" t="s">
         <v>2502</v>
@@ -65478,7 +65481,7 @@
         <v>9</v>
       </c>
       <c r="E45">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F45" t="s">
         <v>2502</v>
@@ -65501,7 +65504,7 @@
         <v>9</v>
       </c>
       <c r="E46">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F46" t="s">
         <v>2502</v>
@@ -65524,7 +65527,7 @@
         <v>9</v>
       </c>
       <c r="E47">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
         <v>2502</v>
@@ -65547,7 +65550,7 @@
         <v>9</v>
       </c>
       <c r="E48">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F48" t="s">
         <v>2502</v>
@@ -65570,7 +65573,7 @@
         <v>9</v>
       </c>
       <c r="E49">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F49" t="s">
         <v>2502</v>
@@ -65593,7 +65596,7 @@
         <v>9</v>
       </c>
       <c r="E50">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F50" t="s">
         <v>2502</v>
@@ -65616,7 +65619,7 @@
         <v>9</v>
       </c>
       <c r="E51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F51" t="s">
         <v>2502</v>
@@ -65639,7 +65642,7 @@
         <v>9</v>
       </c>
       <c r="E52">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F52" t="s">
         <v>2502</v>
@@ -65662,7 +65665,7 @@
         <v>9</v>
       </c>
       <c r="E53">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F53" t="s">
         <v>2502</v>
@@ -65685,7 +65688,7 @@
         <v>9</v>
       </c>
       <c r="E54">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F54" t="s">
         <v>2502</v>
@@ -65708,7 +65711,7 @@
         <v>9</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F55" t="s">
         <v>2502</v>
@@ -65731,7 +65734,7 @@
         <v>9</v>
       </c>
       <c r="E56">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F56" t="s">
         <v>2502</v>
@@ -65754,7 +65757,7 @@
         <v>9</v>
       </c>
       <c r="E57">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F57" t="s">
         <v>2502</v>
@@ -65777,7 +65780,7 @@
         <v>9</v>
       </c>
       <c r="E58">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F58" t="s">
         <v>2502</v>
@@ -65800,7 +65803,7 @@
         <v>9</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F59" t="s">
         <v>2502</v>
@@ -65823,7 +65826,7 @@
         <v>9</v>
       </c>
       <c r="E60">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F60" t="s">
         <v>2502</v>
@@ -65846,7 +65849,7 @@
         <v>9</v>
       </c>
       <c r="E61">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F61" t="s">
         <v>2502</v>
@@ -65869,7 +65872,7 @@
         <v>9</v>
       </c>
       <c r="E62">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F62" t="s">
         <v>2502</v>
@@ -65892,7 +65895,7 @@
         <v>9</v>
       </c>
       <c r="E63">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F63" t="s">
         <v>2502</v>
@@ -65915,7 +65918,7 @@
         <v>9</v>
       </c>
       <c r="E64">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F64" t="s">
         <v>2502</v>
@@ -65938,7 +65941,7 @@
         <v>9</v>
       </c>
       <c r="E65">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F65" t="s">
         <v>2502</v>
@@ -65961,7 +65964,7 @@
         <v>9</v>
       </c>
       <c r="E66">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F66" t="s">
         <v>2502</v>
@@ -65984,7 +65987,7 @@
         <v>9</v>
       </c>
       <c r="E67">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F67" t="s">
         <v>2502</v>
@@ -66007,7 +66010,7 @@
         <v>9</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68" t="s">
         <v>2502</v>
@@ -66030,7 +66033,7 @@
         <v>9</v>
       </c>
       <c r="E69">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F69" t="s">
         <v>2502</v>
@@ -66053,7 +66056,7 @@
         <v>9</v>
       </c>
       <c r="E70">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F70" t="s">
         <v>2502</v>
@@ -66076,7 +66079,7 @@
         <v>9</v>
       </c>
       <c r="E71">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F71" t="s">
         <v>2502</v>
@@ -66122,7 +66125,7 @@
         <v>9</v>
       </c>
       <c r="E73">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F73" t="s">
         <v>2502</v>
@@ -66145,7 +66148,7 @@
         <v>9</v>
       </c>
       <c r="E74">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F74" t="s">
         <v>2502</v>
@@ -66168,7 +66171,7 @@
         <v>9</v>
       </c>
       <c r="E75">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F75" t="s">
         <v>2502</v>
@@ -66191,7 +66194,7 @@
         <v>9</v>
       </c>
       <c r="E76">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F76" t="s">
         <v>2502</v>
@@ -66214,7 +66217,7 @@
         <v>9</v>
       </c>
       <c r="E77">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F77" t="s">
         <v>2502</v>
@@ -66237,7 +66240,7 @@
         <v>9</v>
       </c>
       <c r="E78">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F78" t="s">
         <v>2502</v>
@@ -66260,7 +66263,7 @@
         <v>9</v>
       </c>
       <c r="E79">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F79" t="s">
         <v>2502</v>
@@ -66283,7 +66286,7 @@
         <v>9</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F80" t="s">
         <v>2502</v>
@@ -66306,7 +66309,7 @@
         <v>9</v>
       </c>
       <c r="E81">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F81" t="s">
         <v>2502</v>
@@ -66329,7 +66332,7 @@
         <v>9</v>
       </c>
       <c r="E82">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F82" t="s">
         <v>2502</v>
@@ -66352,7 +66355,7 @@
         <v>9</v>
       </c>
       <c r="E83">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F83" t="s">
         <v>2502</v>
@@ -66375,7 +66378,7 @@
         <v>9</v>
       </c>
       <c r="E84">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F84" t="s">
         <v>2502</v>
@@ -66398,7 +66401,7 @@
         <v>9</v>
       </c>
       <c r="E85">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F85" t="s">
         <v>2502</v>
@@ -66421,7 +66424,7 @@
         <v>9</v>
       </c>
       <c r="E86">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F86" t="s">
         <v>2502</v>
@@ -66444,7 +66447,7 @@
         <v>9</v>
       </c>
       <c r="E87">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F87" t="s">
         <v>2502</v>
@@ -66467,7 +66470,7 @@
         <v>9</v>
       </c>
       <c r="E88">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F88" t="s">
         <v>2502</v>
@@ -66490,7 +66493,7 @@
         <v>9</v>
       </c>
       <c r="E89">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F89" t="s">
         <v>2502</v>
@@ -66513,7 +66516,7 @@
         <v>9</v>
       </c>
       <c r="E90">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F90" t="s">
         <v>2502</v>
@@ -66536,7 +66539,7 @@
         <v>9</v>
       </c>
       <c r="E91">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F91" t="s">
         <v>2502</v>
@@ -66559,7 +66562,7 @@
         <v>9</v>
       </c>
       <c r="E92">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F92" t="s">
         <v>2502</v>
@@ -66582,7 +66585,7 @@
         <v>9</v>
       </c>
       <c r="E93">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F93" t="s">
         <v>2502</v>
@@ -66605,7 +66608,7 @@
         <v>9</v>
       </c>
       <c r="E94">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F94" t="s">
         <v>2502</v>
@@ -66628,7 +66631,7 @@
         <v>9</v>
       </c>
       <c r="E95">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F95" t="s">
         <v>2502</v>
@@ -66651,7 +66654,7 @@
         <v>9</v>
       </c>
       <c r="E96">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F96" t="s">
         <v>2502</v>
@@ -66674,7 +66677,7 @@
         <v>9</v>
       </c>
       <c r="E97">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F97" t="s">
         <v>2502</v>
@@ -66697,7 +66700,7 @@
         <v>9</v>
       </c>
       <c r="E98">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F98" t="s">
         <v>2502</v>
@@ -66720,7 +66723,7 @@
         <v>9</v>
       </c>
       <c r="E99">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F99" t="s">
         <v>2502</v>
@@ -66766,7 +66769,7 @@
         <v>9</v>
       </c>
       <c r="E101">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F101" t="s">
         <v>2502</v>
@@ -66789,7 +66792,7 @@
         <v>9</v>
       </c>
       <c r="E102">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F102" t="s">
         <v>2502</v>
@@ -66812,7 +66815,7 @@
         <v>9</v>
       </c>
       <c r="E103">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F103" t="s">
         <v>2502</v>
@@ -66835,7 +66838,7 @@
         <v>9</v>
       </c>
       <c r="E104">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F104" t="s">
         <v>2502</v>
@@ -66858,7 +66861,7 @@
         <v>9</v>
       </c>
       <c r="E105">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F105" t="s">
         <v>2502</v>
@@ -66881,7 +66884,7 @@
         <v>9</v>
       </c>
       <c r="E106">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F106" t="s">
         <v>2502</v>
@@ -66904,7 +66907,7 @@
         <v>9</v>
       </c>
       <c r="E107">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F107" t="s">
         <v>2502</v>
@@ -66927,7 +66930,7 @@
         <v>9</v>
       </c>
       <c r="E108">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F108" t="s">
         <v>2502</v>
@@ -66950,7 +66953,7 @@
         <v>9</v>
       </c>
       <c r="E109">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="F109" t="s">
         <v>2502</v>
@@ -66973,7 +66976,7 @@
         <v>9</v>
       </c>
       <c r="E110">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F110" t="s">
         <v>2502</v>
@@ -66996,7 +66999,7 @@
         <v>9</v>
       </c>
       <c r="E111">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F111" t="s">
         <v>2502</v>
@@ -67019,7 +67022,7 @@
         <v>9</v>
       </c>
       <c r="E112">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F112" t="s">
         <v>2502</v>
@@ -67042,7 +67045,7 @@
         <v>9</v>
       </c>
       <c r="E113">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F113" t="s">
         <v>2502</v>
@@ -67065,7 +67068,7 @@
         <v>9</v>
       </c>
       <c r="E114">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F114" t="s">
         <v>2502</v>
@@ -67088,7 +67091,7 @@
         <v>9</v>
       </c>
       <c r="E115">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F115" t="s">
         <v>2502</v>
@@ -67111,7 +67114,7 @@
         <v>9</v>
       </c>
       <c r="E116">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F116" t="s">
         <v>2502</v>
@@ -67180,7 +67183,7 @@
         <v>9</v>
       </c>
       <c r="E119">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F119" t="s">
         <v>2502</v>
@@ -67203,7 +67206,7 @@
         <v>9</v>
       </c>
       <c r="E120">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F120" t="s">
         <v>2502</v>

</xml_diff>